<commit_message>
Forms sync auto batch 4: 5000 files
</commit_message>
<xml_diff>
--- a/file_upload_forms/047_environmental_fieldwork_documentation_release_form--file_upload_forms.xlsx
+++ b/file_upload_forms/047_environmental_fieldwork_documentation_release_form--file_upload_forms.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -642,8 +642,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
-    <col width="33" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -671,12 +671,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{'name':_'yes',_'value':_'yes'}</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{'name': 'Yes', 'value': 'Yes'}</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -688,12 +688,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{'name':_'no',_'value':_'no'}</t>
+          <t>no</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{'name': 'No', 'value': 'No'}</t>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>